<commit_message>
fix hstroke RRi bug
</commit_message>
<xml_diff>
--- a/data/processed/ettehad_rr_bp_reduction_effects_bplttc_2021.xlsx
+++ b/data/processed/ettehad_rr_bp_reduction_effects_bplttc_2021.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/02Work/WHO-CVD/github/uw-who-cvdtargets/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="8_{331CF8A5-94EE-488E-B7B7-4C4AC6851445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{296BC16C-FEA6-47DC-87A5-3F25ABDFF457}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="8_{331CF8A5-94EE-488E-B7B7-4C4AC6851445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5014539F-2C96-4BE7-94A9-F55BAA2BAC0E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ACAEEDB5-3BB2-45B3-B3BF-2A292CDA7EEB}"/>
   </bookViews>
@@ -884,7 +884,7 @@
     <col min="7" max="7" width="18.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="43.8" thickBot="1">
+    <row r="1" spans="1:9" ht="29.4" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2205,15 +2205,15 @@
         <v>0.87</v>
       </c>
       <c r="F2" s="39">
-        <f>+C2^2</f>
+        <f t="shared" ref="F2:H3" si="0">+C2^2</f>
         <v>0.6241000000000001</v>
       </c>
       <c r="G2" s="32">
-        <f>+D2^2</f>
+        <f t="shared" si="0"/>
         <v>0.51839999999999997</v>
       </c>
       <c r="H2" s="32">
-        <f>+E2^2</f>
+        <f t="shared" si="0"/>
         <v>0.75690000000000002</v>
       </c>
       <c r="I2" s="31" t="s">
@@ -2237,15 +2237,15 @@
         <v>0.98</v>
       </c>
       <c r="F3" s="39">
-        <f>+C3^2</f>
+        <f t="shared" si="0"/>
         <v>0.82810000000000006</v>
       </c>
       <c r="G3" s="32">
-        <f>+D3^2</f>
+        <f t="shared" si="0"/>
         <v>0.72249999999999992</v>
       </c>
       <c r="H3" s="32">
-        <f>+E3^2</f>
+        <f t="shared" si="0"/>
         <v>0.96039999999999992</v>
       </c>
       <c r="I3" s="33" t="s">
@@ -2269,15 +2269,15 @@
         <v>0.99</v>
       </c>
       <c r="F4" s="39">
-        <f t="shared" ref="F4:F43" si="0">+C4^2</f>
+        <f t="shared" ref="F4:F43" si="1">+C4^2</f>
         <v>0.88359999999999994</v>
       </c>
       <c r="G4" s="32">
-        <f t="shared" ref="G4:G43" si="1">+D4^2</f>
+        <f t="shared" ref="G4:G43" si="2">+D4^2</f>
         <v>0.79210000000000003</v>
       </c>
       <c r="H4" s="32">
-        <f t="shared" ref="H4:H43" si="2">+E4^2</f>
+        <f t="shared" ref="H4:H43" si="3">+E4^2</f>
         <v>0.98009999999999997</v>
       </c>
       <c r="I4" s="33" t="s">
@@ -2301,15 +2301,15 @@
         <v>0.98</v>
       </c>
       <c r="F5" s="39">
-        <f t="shared" si="0"/>
+        <f>+C5^2</f>
         <v>0.86490000000000011</v>
       </c>
       <c r="G5" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="H5" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.96039999999999992</v>
       </c>
       <c r="I5" s="33" t="s">
@@ -2333,15 +2333,15 @@
         <v>0.94</v>
       </c>
       <c r="F6" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="G6" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.68889999999999996</v>
       </c>
       <c r="H6" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.88359999999999994</v>
       </c>
       <c r="I6" s="33" t="s">
@@ -2365,15 +2365,15 @@
         <v>0.92</v>
       </c>
       <c r="F7" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.75690000000000002</v>
       </c>
       <c r="G7" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.68889999999999996</v>
       </c>
       <c r="H7" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.84640000000000004</v>
       </c>
       <c r="I7" s="33" t="s">
@@ -2397,15 +2397,15 @@
         <v>0.94</v>
       </c>
       <c r="F8" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.81</v>
       </c>
       <c r="G8" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.73959999999999992</v>
       </c>
       <c r="H8" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.88359999999999994</v>
       </c>
       <c r="I8" s="33" t="s">
@@ -2429,15 +2429,15 @@
         <v>0.97</v>
       </c>
       <c r="F9" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.6241000000000001</v>
       </c>
       <c r="G9" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.42250000000000004</v>
       </c>
       <c r="H9" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.94089999999999996</v>
       </c>
       <c r="I9" s="33" t="s">
@@ -2461,15 +2461,15 @@
         <v>0.99</v>
       </c>
       <c r="F10" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.73959999999999992</v>
       </c>
       <c r="G10" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.54759999999999998</v>
       </c>
       <c r="H10" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.98009999999999997</v>
       </c>
       <c r="I10" s="33" t="s">
@@ -2493,15 +2493,15 @@
         <v>1.02</v>
       </c>
       <c r="F11" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.84640000000000004</v>
       </c>
       <c r="G11" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.68889999999999996</v>
       </c>
       <c r="H11" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0404</v>
       </c>
       <c r="I11" s="33" t="s">
@@ -2525,15 +2525,15 @@
         <v>0.99</v>
       </c>
       <c r="F12" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.81</v>
       </c>
       <c r="G12" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.67239999999999989</v>
       </c>
       <c r="H12" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.98009999999999997</v>
       </c>
       <c r="I12" s="33" t="s">
@@ -2557,15 +2557,15 @@
         <v>0.92</v>
       </c>
       <c r="F13" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.59289999999999998</v>
       </c>
       <c r="G13" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.42250000000000004</v>
       </c>
       <c r="H13" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.84640000000000004</v>
       </c>
       <c r="I13" s="33" t="s">
@@ -2589,15 +2589,15 @@
         <v>0.94</v>
       </c>
       <c r="F14" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.73959999999999992</v>
       </c>
       <c r="G14" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.6241000000000001</v>
       </c>
       <c r="H14" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.88359999999999994</v>
       </c>
       <c r="I14" s="33" t="s">
@@ -2621,15 +2621,15 @@
         <v>0.97</v>
       </c>
       <c r="F15" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.81</v>
       </c>
       <c r="G15" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.70559999999999989</v>
       </c>
       <c r="H15" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.94089999999999996</v>
       </c>
       <c r="I15" s="33" t="s">
@@ -2653,15 +2653,15 @@
         <v>0.95</v>
       </c>
       <c r="F16" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.68889999999999996</v>
       </c>
       <c r="G16" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.51839999999999997</v>
       </c>
       <c r="H16" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.90249999999999997</v>
       </c>
       <c r="I16" s="33" t="s">
@@ -2685,15 +2685,15 @@
         <v>1.05</v>
       </c>
       <c r="F17" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.90249999999999997</v>
       </c>
       <c r="G17" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.73959999999999992</v>
       </c>
       <c r="H17" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1025</v>
       </c>
       <c r="I17" s="33" t="s">
@@ -2717,15 +2717,15 @@
         <v>1.04</v>
       </c>
       <c r="F18" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.92159999999999997</v>
       </c>
       <c r="G18" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="H18" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0816000000000001</v>
       </c>
       <c r="I18" s="33" t="s">
@@ -2749,15 +2749,15 @@
         <v>1.02</v>
       </c>
       <c r="F19" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.88359999999999994</v>
       </c>
       <c r="G19" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.75690000000000002</v>
       </c>
       <c r="H19" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0404</v>
       </c>
       <c r="I19" s="33" t="s">
@@ -2781,15 +2781,15 @@
         <v>0.99</v>
       </c>
       <c r="F20" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.82810000000000006</v>
       </c>
       <c r="G20" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.68889999999999996</v>
       </c>
       <c r="H20" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.98009999999999997</v>
       </c>
       <c r="I20" s="33" t="s">
@@ -2813,15 +2813,15 @@
         <v>0.95</v>
       </c>
       <c r="F21" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.75690000000000002</v>
       </c>
       <c r="G21" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.64000000000000012</v>
       </c>
       <c r="H21" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.90249999999999997</v>
       </c>
       <c r="I21" s="33" t="s">
@@ -2845,15 +2845,15 @@
         <v>1.01</v>
       </c>
       <c r="F22" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.88359999999999994</v>
       </c>
       <c r="G22" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="H22" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0201</v>
       </c>
       <c r="I22" s="33" t="s">
@@ -2877,15 +2877,15 @@
         <v>0.96</v>
       </c>
       <c r="F23" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.60840000000000005</v>
       </c>
       <c r="G23" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.40960000000000002</v>
       </c>
       <c r="H23" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.92159999999999997</v>
       </c>
       <c r="I23" s="33" t="s">
@@ -2909,15 +2909,15 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="F24" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.98009999999999997</v>
       </c>
       <c r="G24" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.72249999999999992</v>
       </c>
       <c r="H24" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.3224999999999998</v>
       </c>
       <c r="I24" s="33" t="s">
@@ -2941,15 +2941,15 @@
         <v>0.97</v>
       </c>
       <c r="F25" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.72249999999999992</v>
       </c>
       <c r="G25" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.5625</v>
       </c>
       <c r="H25" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.94089999999999996</v>
       </c>
       <c r="I25" s="33" t="s">
@@ -2973,15 +2973,15 @@
         <v>1.07</v>
       </c>
       <c r="F26" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.90249999999999997</v>
       </c>
       <c r="G26" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.72249999999999992</v>
       </c>
       <c r="H26" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1449</v>
       </c>
       <c r="I26" s="33" t="s">
@@ -3005,15 +3005,15 @@
         <v>1</v>
       </c>
       <c r="F27" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="G27" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.60840000000000005</v>
       </c>
       <c r="H27" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="I27" s="33" t="s">
@@ -3037,15 +3037,15 @@
         <v>0.8</v>
       </c>
       <c r="F28" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.48999999999999994</v>
       </c>
       <c r="G28" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.37209999999999999</v>
       </c>
       <c r="H28" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.64000000000000012</v>
       </c>
       <c r="I28" s="33" t="s">
@@ -3069,15 +3069,15 @@
         <v>1</v>
       </c>
       <c r="F29" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.79210000000000003</v>
       </c>
       <c r="G29" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.6241000000000001</v>
       </c>
       <c r="H29" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="I29" s="33" t="s">
@@ -3101,15 +3101,15 @@
         <v>1.1200000000000001</v>
       </c>
       <c r="F30" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.81</v>
       </c>
       <c r="G30" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.51839999999999997</v>
       </c>
       <c r="H30" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.2544000000000002</v>
       </c>
       <c r="I30" s="33" t="s">
@@ -3133,15 +3133,15 @@
         <v>1.05</v>
       </c>
       <c r="F31" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.79210000000000003</v>
       </c>
       <c r="G31" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.5776</v>
       </c>
       <c r="H31" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1025</v>
       </c>
       <c r="I31" s="33" t="s">
@@ -3165,15 +3165,15 @@
         <v>1.1100000000000001</v>
       </c>
       <c r="F32" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.96039999999999992</v>
       </c>
       <c r="G32" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.75690000000000002</v>
       </c>
       <c r="H32" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.2321000000000002</v>
       </c>
       <c r="I32" s="33" t="s">
@@ -3197,15 +3197,15 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="F33" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.94089999999999996</v>
       </c>
       <c r="G33" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.73959999999999992</v>
       </c>
       <c r="H33" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.2100000000000002</v>
       </c>
       <c r="I33" s="33" t="s">
@@ -3229,15 +3229,15 @@
         <v>1.1399999999999999</v>
       </c>
       <c r="F34" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G34" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="H34" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.2995999999999999</v>
       </c>
       <c r="I34" s="33" t="s">
@@ -3261,15 +3261,15 @@
         <v>0.99</v>
       </c>
       <c r="F35" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.81</v>
       </c>
       <c r="G35" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.67239999999999989</v>
       </c>
       <c r="H35" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.98009999999999997</v>
       </c>
       <c r="I35" s="33" t="s">
@@ -3293,15 +3293,15 @@
         <v>1.02</v>
       </c>
       <c r="F36" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.90249999999999997</v>
       </c>
       <c r="G36" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="H36" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0404</v>
       </c>
       <c r="I36" s="33" t="s">
@@ -3325,15 +3325,15 @@
         <v>1</v>
       </c>
       <c r="F37" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="G37" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.60840000000000005</v>
       </c>
       <c r="H37" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="I37" s="33" t="s">
@@ -3357,15 +3357,15 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="F38" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G38" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.82810000000000006</v>
       </c>
       <c r="H38" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.2100000000000002</v>
       </c>
       <c r="I38" s="33" t="s">
@@ -3389,15 +3389,15 @@
         <v>1.05</v>
       </c>
       <c r="F39" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.96039999999999992</v>
       </c>
       <c r="G39" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.82810000000000006</v>
       </c>
       <c r="H39" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1025</v>
       </c>
       <c r="I39" s="33" t="s">
@@ -3421,15 +3421,15 @@
         <v>1.06</v>
       </c>
       <c r="F40" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.98009999999999997</v>
       </c>
       <c r="G40" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.84640000000000004</v>
       </c>
       <c r="H40" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1236000000000002</v>
       </c>
       <c r="I40" s="33" t="s">
@@ -3453,15 +3453,15 @@
         <v>1.07</v>
       </c>
       <c r="F41" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.90249999999999997</v>
       </c>
       <c r="G41" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.72249999999999992</v>
       </c>
       <c r="H41" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1449</v>
       </c>
       <c r="I41" s="33" t="s">
@@ -3485,15 +3485,15 @@
         <v>1</v>
       </c>
       <c r="F42" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.88359999999999994</v>
       </c>
       <c r="G42" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.77439999999999998</v>
       </c>
       <c r="H42" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="I42" s="33" t="s">
@@ -3517,15 +3517,15 @@
         <v>1.02</v>
       </c>
       <c r="F43" s="39">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.94089999999999996</v>
       </c>
       <c r="G43" s="32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.86490000000000011</v>
       </c>
       <c r="H43" s="32">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0404</v>
       </c>
       <c r="I43" s="35" t="s">

</xml_diff>